<commit_message>
feat: implement paginated scraping and deduplication for LinkedIn and Indeed job portals
</commit_message>
<xml_diff>
--- a/scraped_jobs_permanent.xlsx
+++ b/scraped_jobs_permanent.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,22 +461,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>.NET Developer</t>
+          <t>Full Stack .Net Developer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NonStop io Technologies</t>
+          <t>Iris Software</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hybrid - Pune, Noida, Gurugram</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/jobs/view/net-developer-at-nonstop-io-technologies-4431948397</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-iris-software-noida-pune-gurugram-5-to-9-years-101225025922</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,22 +503,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lead C# .NET Developer (Windows Services &amp; Desktop UI)</t>
+          <t>.Net developer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Williams-Sonoma, Inc.</t>
+          <t>Xoriant</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hybrid - Pune, Bengaluru, Mumbai (All Areas)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/jobs/view/lead-c%23-net-developer-windows-services-desktop-ui-at-williams-sonoma-inc-4367152383</t>
+          <t>https://www.naukri.com/job-listings-net-developer-xoriant-pune-bengaluru-mumbai-all-areas-5-to-10-years-080926016033</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -545,22 +545,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>.NET DEVELOPER – OPERATIONS &amp; SUPPORT (HOSPITALITY)</t>
+          <t>Full Stack .Net Developer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Zensar Technologies</t>
+          <t>Cloudxtreme</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/jobs/view/net-developer-%E2%80%93-operations-support-hospitality-at-zensar-technologies-4434144245</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-cloudxtreme-pune-6-to-11-years-040926927741</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -587,22 +587,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TCS Hiring | Azure .Net Developers | Pune(Face to Face Interview) | 4th July 2026</t>
+          <t>Senior .Net Developer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services</t>
+          <t>TEKsystems</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hybrid - Pune</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/jobs/view/tcs-hiring-azure-net-developers-pune-face-to-face-interview-4th-july-2026-at-tata-consultancy-services-4432980382</t>
+          <t>https://www.naukri.com/job-listings-senior-net-developer-allegis-group-pune-5-to-8-years-310826027339</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,22 +629,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Senior Analyst Developer (Senior .NET Developer)</t>
+          <t>Full Stack .NET Developer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FNZ</t>
+          <t>A.P. Moller Maersk</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://in.linkedin.com/jobs/view/senior-analyst-developer-senior-net-developer-at-fnz-4432327757</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-a-p-moller-maersk-pune-3-to-5-years-310826009438</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -671,32 +671,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Full Stack .Net Developer-S</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hybrid - Pune, Chennai, Bengaluru</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=237ac399c7c99b10&amp;bb=2Q2I2vS5IVwe9-2s60xDz5iGEVbmzlkcgSLL6tYiNkyWqzXe50eh6iMT2-mEXgGHfPj06TGAAdfZAU-y0KI7GFNQFtMZxYb3fXXKDF5HFp0gpqmQsGw29WTIFTjxfNVHbsyrig8y2Vb3RTlM6K6nIfEKoxdPJu2D&amp;xkcb=SoDy67M3hW_TkWzDMp0LbzkdCdPP&amp;fccid=50186c24e94ffd1a&amp;cmp=Amshoft-IT-Solution&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-s-infosys-pune-chennai-bengaluru-2-to-3-years-100826024367</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -713,32 +713,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>dot net,.NET developer Angular</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cloudxtreme</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hybrid - Pune, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=237ac399c7c99b10&amp;bb=2Q2I2vS5IVwe9-2s60xDz5iGEVbmzlkcgSLL6tYiNkyWqzXe50eh6iMT2-mEXgGHfPj06TGAAdfZAU-y0KI7GFNQFtMZxYb3fXXKDF5HFp0gpqmQsGw29WTIFTjxfNVHbsyrig8y2Vb3RTlM6K6nIfEKoxdPJu2D&amp;xkcb=SoDy67M3hW_TkWzDMp0LbzkdCdPP&amp;fccid=50186c24e94ffd1a&amp;cmp=Amshoft-IT-Solution&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-dot-net-net-developer-angular-cloudxtreme-hyderabad-pune-bengaluru-9-to-14-years-040926927136</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -755,32 +755,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>ASP .NET developer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Cloudxtreme</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune, Bengaluru</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=51c964be2082f5e4&amp;bb=2Q2I2vS5IVwe9-2s60xDzz9KiT9OgE0dvcYqGkaXyqNLz0Ro1QpJYPwroKcf_nw6xaLgCT96b7shut-2yncdXmsVbBwRNu47BEbskCcymIlJouZcFVGlI_ASDdOct_VMlbp9MVghxh8x9EUlpxeppLrKpvyn_0Au&amp;xkcb=SoBG67M3hW_TkWzDMp0KbzkdCdPP&amp;fccid=dd5dd1e5293634a3&amp;cmp=AV-SoftTech&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-asp-net-developer-cloudxtreme-pune-bengaluru-8-to-12-years-040926922418</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -797,32 +797,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.NET Developer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Iris Software</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hybrid - Pune, Noida, Gurugram</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=51c964be2082f5e4&amp;bb=2Q2I2vS5IVwe9-2s60xDzz9KiT9OgE0dvcYqGkaXyqNLz0Ro1QpJYPwroKcf_nw6xaLgCT96b7shut-2yncdXmsVbBwRNu47BEbskCcymIlJouZcFVGlI_ASDdOct_VMlbp9MVghxh8x9EUlpxeppLrKpvyn_0Au&amp;xkcb=SoBG67M3hW_TkWzDMp0KbzkdCdPP&amp;fccid=dd5dd1e5293634a3&amp;cmp=AV-SoftTech&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-net-developer-iris-software-noida-pune-gurugram-7-to-9-years-030826007974</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -839,32 +839,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Full Stack .Net Developer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Ascendion Engineering Private Limited</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hybrid - Pune, Chennai, Bengaluru</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=450718eae0c08c88&amp;bb=2Q2I2vS5IVwe9-2s60xDz2AvMYQg3KK7hoCj9E5-YgAPblplx56ySVuIKmKCx4FSBXe3GQRCV-BZ1e65z5_eYM1UQlDxjTSqYFN2432OtuWMMiviRXltM90oi4HLej1eJBsbN6hL7tnsyuukAVaES-GE43aLMCNj&amp;xkcb=SoDb67M3hW_TkWzDMp0JbzkdCdPP&amp;fccid=dc1449c6fe744ee9&amp;cmp=Kasmoprav&amp;ti=Full+Stack+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-ascendion-engineering-pune-chennai-bengaluru-6-to-11-years-290826011186</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -881,32 +881,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net developer @Pan India</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hybrid - Pune, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=450718eae0c08c88&amp;bb=2Q2I2vS5IVwe9-2s60xDz2AvMYQg3KK7hoCj9E5-YgAPblplx56ySVuIKmKCx4FSBXe3GQRCV-BZ1e65z5_eYM1UQlDxjTSqYFN2432OtuWMMiviRXltM90oi4HLej1eJBsbN6hL7tnsyuukAVaES-GE43aLMCNj&amp;xkcb=SoDb67M3hW_TkWzDMp0JbzkdCdPP&amp;fccid=dc1449c6fe744ee9&amp;cmp=Kasmoprav&amp;ti=Full+Stack+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-net-developer-pan-india-infosys-hyderabad-pune-bengaluru-3-to-5-years-280826002353</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -923,32 +923,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net developer @Pan India</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Hybrid - Pune, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=f3c6f2f935648768&amp;bb=2Q2I2vS5IVwe9-2s60xDzzeH9SOBchK9mgEzVG8gm5WuM0yKJTJgTVoLuEziReLmzhJi-9qW9gHnNI5-INrcXXjxeH2JIxTva6-VOuRzbAkz8cHDo1VCwdKm2rg0sBSw8hIsBorBV3y4cUXD5mX408N29Jc6OOen&amp;xkcb=SoBv67M3hW_TkWzDMp0IbzkdCdPP&amp;fccid=5f02de3877c7cf9c&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-net-developer-pan-india-infosys-hyderabad-pune-bengaluru-3-to-5-years-270826012518</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -965,32 +965,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Full Stack .Net Developer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Technossus Software Services</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune, Ludhiana, Chandigarh</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=f3c6f2f935648768&amp;bb=2Q2I2vS5IVwe9-2s60xDzzeH9SOBchK9mgEzVG8gm5WuM0yKJTJgTVoLuEziReLmzhJi-9qW9gHnNI5-INrcXXjxeH2JIxTva6-VOuRzbAkz8cHDo1VCwdKm2rg0sBSw8hIsBorBV3y4cUXD5mX408N29Jc6OOen&amp;xkcb=SoBv67M3hW_TkWzDMp0IbzkdCdPP&amp;fccid=5f02de3877c7cf9c&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-technossus-software-services-ludhiana-chandigarh-pune-5-to-10-years-260826017336</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1007,32 +1007,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Naukri</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Full Stack .Net Developer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Xoriant</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune, Hyderabad, Bengaluru</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3+ years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/rc/clk?jk=8ad932df2d5416bd&amp;bb=2Q2I2vS5IVwe9-2s60xDz3segUpq3dovGyv856fo5zofhlvjlDX23BPNaXpDUIWeAyDP6X-7TB4YCF3gwBhkqSkyOAG3u9iX3vlYcmWR_RTUzQWDDkRrTRc1kYAu50AWisdBpnekaXj0vs4K5XBvSH_XfZVFbsgn&amp;xkcb=SoDh67M3hW_TkWzDMp0PbzkdCdPP&amp;fccid=dd616958bd9ddc12&amp;cmp=Mobicloud&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.naukri.com/job-listings-full-stack-net-developer-xoriant-hyderabad-pune-bengaluru-5-to-9-years-240326010337</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1049,40 +1049,2224 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Coditas</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/net-developer-at-coditas-4461573520</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>C# .Net Developer</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cavista Technologies</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/c%23-net-developer-at-cavista-technologies-4464998185</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lead C# .NET Developer (Windows Services &amp; Desktop UI)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Williams-Sonoma, Inc.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/lead-c%23-net-developer-windows-services-desktop-ui-at-williams-sonoma-inc-4367152383</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>.Net Developer, AS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/net-developer-as-at-deutsche-bank-4464402683</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Senior Full Stack .NET Developer (F/M/D)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Freudenberg Filtration Technologies</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-full-stack-net-developer-f-m-d-at-freudenberg-filtration-technologies-4461092197</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C# .NET Developer</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/c-net-developer-persistent-systems-JV_IC2856202_KO0,15_KE16,34.htm?jl=1010242140132</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Asp .Net Developer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Vision Cloud</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/asp-net-developer-vision-cloud-JV_IC2856202_KO0,17_KE18,30.htm?jl=1007660714907</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>IT Shastra</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-it-shastra-JV_IC2856202_KO0,13_KE14,24.htm?jl=1010106159756</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ASP .NET Developer</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CDAT Pune</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/asp-net-developer-cdat-pune-JV_IC2856202_KO0,17_KE18,27.htm?jl=1010161349511</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MDI NetworX</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-mdi-networx-JV_IC2856202_KO0,13_KE14,25.htm?jl=1010065634540</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C# .Net Developer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Leuwint Technologies,</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/c-net-developer-leuwint-technologies-JV_IC2856202_KO0,15_KE16,36.htm?jl=1010199488605</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>.Net Developer, AS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Deutsche Bank</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-as-deutsche-bank-JV_IC2856202_KO0,16_KE17,30.htm?jl=1010088302927</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Junior .Net Developer</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Komax Group</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/junior-net-developer-komax-group-JV_IC2856202_KO0,20_KE21,32.htm?jl=1010159269310</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mechatronics Systems</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-mechatronics-systems-JV_IC2856202_KO0,13_KE14,34.htm?jl=1008234944903</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>.NET developer ( Associate Software)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>HOERBIGER</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-associate-software-hoerbiger-JV_IC2856202_KO0,32_KE33,42.htm?jl=1010205323457</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>.NET Developer</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-persistent-systems-JV_IC2856202_KO0,13_KE14,32.htm?jl=1010229099114</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Paratus Systems</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-paratus-systems-JV_IC2856202_KO0,13_KE14,29.htm?jl=1006581616911</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Triotech Software System</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-triotech-software-system-JV_IC2856202_KO0,13_KE14,38.htm?jl=1007872878984</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>.Net developer</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Elysiar Technologies</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-elysiar-technologies-JV_IC2856202_KO0,13_KE14,34.htm?jl=1006887054899</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>.NET Developer</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Siddhatech Software Services</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-siddhatech-software-services-JV_IC2856202_KO0,13_KE14,42.htm?jl=1005897504638</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>www.placementindia.com</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Apply to 118 .Net Developer Job Vacancies in Pune</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>www.placementindia.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.placementindia.com/job-search/full-stack-web-developer-jobs-in-pune.htm</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>.Net Developer5 - 7 yrsMumbai.Net.Net CoreC#ASPPosted 1 week agoPosted 1 week ago</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-1667585?ref=sp&amp;jobPos=2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>.Net Developer - ASP/MVC5 - 10 yrsBangalore4.324+ Reviews.NetBackend ArchitectureASPMVC.Net CoreC#+1Posted 1 day agoPosted 1 day ago</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-asp-mvc-1669727?ref=sp&amp;jobPos=3</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>.Net Developer - C# Programming4 - 7 yrsNoidaC#.NetBackend ArchitectureDesign PatternsSQL ServerPosted 1 week agoPosted 1 week ago</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-programming-1667662?ref=sp&amp;jobPos=4</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>.Net Developer - Backend Architecture3 - 6 yrsMultiple LocationsC#.Net Core.NetEntity FrameworkBackend ArchitecturePosted 1 week agoPosted 1 week ago</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-backend-architecture-1667093?ref=sp&amp;jobPos=6</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>.Net Developer5 - 10 yrsBangalore/Chennai/Mysore.NetC#ASP.Net CoreWebAPIAzureMicroservices Architecture+2Posted 2 weeks agoPosted 2 weeks ago</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-1664767?ref=sp&amp;jobPos=7</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>.Net Developer - C#/ASP/WebAPI5 - 10 yrs15-35 LPABangalore4.324+ Reviews.NetC#ASPMicroservices ArchitectureEntity FrameworkPosted 1 week agoPosted 1 week ago</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-asp-webapi-1666897?ref=sp&amp;jobPos=8</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>.Net Developer - ASP/C#5 - 7 yrsKarnataka.Net.Net CoreC#ASPSQL ServerOOPSMVC+2Posted 2 weeks agoPosted 2 weeks ago</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-asp-c-1665983?ref=sp&amp;jobPos=9</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Senior .Net Developer5 - 10 yrsPune/Chennai/Bangalore4.518+ Reviews.Net.Net CoreASPSQL ServerC#WCFADOBlazorMicroservices Architecture+4Posted 1 week agoPosted 1 week ago</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/senior-net-developer-1668110?ref=sp&amp;jobPos=11</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>.Net Developer - ASP/MVC5 - 10 yrsPune/Jaipur.Net.Net CoreMVCSQL ServerEntity FrameworkASP+1Posted 2 weeks agoPosted 2 weeks ago</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-asp-mvc-1665238?ref=sp&amp;jobPos=12</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>.Net Developer4 - 5 yrsGurgaon/Gurugram.Net.Net CoreC#ASPSQL ServerPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-1661699?ref=sp&amp;jobPos=13</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Senior .Net Developer10 - 15 yrsOverseas/International.NetC#.Net CorePosted 2 weeks agoPosted 2 weeks ago</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/senior-net-developer-1665373?ref=sp&amp;jobPos=15</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>.Net Developer - Microservices Architecture5 - 8 yrsMultiple Locations53+ ReviewsMay work from home.NetMicroservices Architecture.Net CorePosted 4 weeks agoPosted 4 weeks ago</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-microservices-architecture-1662395?ref=sp&amp;jobPos=16</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BDO India LLP - .Net Developer - Kentico4 - 10 yrsAny Location.NetKentico.Net CoreC#ASPPosted 3 weeks agoPosted 3 weeks ago</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/bdo-india-llp-net-developer-kentico-1663779?ref=sp&amp;jobPos=17</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Senior .Net Developer - C#/ASP10 - 15 yrsDubai/Overseas/International.NetMicroservices ArchitectureSQL ServerASPC#Posted 1 week agoPosted 1 week ago</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/senior-net-developer-c-asp-1666637?ref=sp&amp;jobPos=18</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>.Net Developer - C#/ASP4 - 6 yrsGurgaon/GurugramBackend Architecture.NetC#.Net CoreASPPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-asp-1661615?ref=sp&amp;jobPos=19</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Indeed</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>3+ years</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://www.indeed.com/rc/clk?jk=8ad932df2d5416bd&amp;bb=2Q2I2vS5IVwe9-2s60xDz3segUpq3dovGyv856fo5zofhlvjlDX23BPNaXpDUIWeAyDP6X-7TB4YCF3gwBhkqSkyOAG3u9iX3vlYcmWR_RTUzQWDDkRrTRc1kYAu50AWisdBpnekaXj0vs4K5XBvSH_XfZVFbsgn&amp;xkcb=SoDh67M3hW_TkWzDMp0PbzkdCdPP&amp;fccid=dd616958bd9ddc12&amp;cmp=Mobicloud&amp;ti=.NET+Developer&amp;vjs=3</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Refer to Apply Link</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=c3cefe92e87022b3&amp;bb=ez91sI_i5AG6dZ3D-oMOPl97Tu5QMQObtsUeIap4xTx9CwtVZrTGLX-Hlu7zk5fWGBtPzJ-fc7cKfpQrn9zGVB89W1U7K844FqSn1zHiCCoPaOr356tMg7ws7DxB7hLH&amp;xkcb=SoCr67M2eDlWVygfKz0LbzkdCdPP&amp;fccid=ea6bb53f0b18b8f2&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=a39baff881378c7e&amp;bb=ez91sI_i5AG6dZ3D-oMOPsAw_OIjF2fkPDNoKRLoJqgqlXcq5jE7B5gsbeP0Jc2HycqCWMmdWhWOiYqv7hSqeTHmxdZjIA0xJWWk7pfh5dStoWUK_PCvy4e_KOS9Js88&amp;xkcb=SoAf67M2eDlWVygfKz0KbzkdCdPP&amp;fccid=b90433ed96d63887&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=d801945573fc49b3&amp;bb=ez91sI_i5AG6dZ3D-oMOPp24p5ozE1b8Zvh8_RT5WHiwVTEqUG4R92CkeRcs4qFcuVNCSmO2CxZIS7_AQsg09H2t8IpXLBktdHq-ZuwczCaN5b3OZGrlw4gANb7zonRo&amp;xkcb=SoCC67M2eDlWVygfKz0JbzkdCdPP&amp;fccid=044454a3614573b1&amp;cmp=Kognivera-IT-Solutions&amp;ti=Full+Stack+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=16e264233fd534be&amp;bb=ez91sI_i5AG6dZ3D-oMOPmngYtHU0_TKPq-V-uF7FSNlDLKn_1sRPFSXNDZgNDrnS3hJoUe2_kgc0hfX1QOBk0eY0iGAjalt2cq8NnSJ3CC0N9ChSsJ7z4zEJXqAFzWX&amp;xkcb=SoA267M2eDlWVygfKz0IbzkdCdPP&amp;fccid=e70d0cb4e4e9ff3e&amp;cmp=Mobileprogramming&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=23e7f16e85a6051c&amp;bb=ez91sI_i5AG6dZ3D-oMOPrcgI4Nhak993NFj0eobi4vhP5Ncmb2-DE1gHJKtZUbx2Rvm6KHoqpwtJ2yNlLuyBwEdXODk9_paEqnAKv6Ic_7bMADgKQbfz1Rm16cpwr_W&amp;xkcb=SoC467M2eDlWVygfKz0PbzkdCdPP&amp;fccid=3974499deb2a6701&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=7a84c94472b5bf08&amp;bb=ez91sI_i5AG6dZ3D-oMOPi42bUHUYcNGz4_F4OQZx4h3bJVG5UBC0nSretkDvkfFE6P3EBat4z8uTAxBt_Mi6qb6pAHVSvNOmLJJ-8hSPNprQqLz4p-1EhbDxXwRR9N8&amp;xkcb=SoAM67M2eDlWVygfKz0ObzkdCdPP&amp;fccid=0140e51652b12787&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=8c16379eaeec7da7&amp;bb=ez91sI_i5AG6dZ3D-oMOPnZxRhz_jWPJY0oNiwir9l2t0C7QqJWEsMmLaoFeW9FnEAP6yA4XgOwlbxNUrtKEQlzS0SVXxQB95hNv7lKUV_ZJYfGOsWOSAsZyNegcvI-L&amp;xkcb=SoCR67M2eDlWVygfKz0NbzkdCdPP&amp;fccid=059470e192337a9a&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=ec1a91d090fc5539&amp;bb=ez91sI_i5AG6dZ3D-oMOPoEalpxfwO1FSNTn_zbtlGz_ol_fpKKlYLhPHO-eL8QWRIe0cPNRVVCiJbV2E8PXyYyHsDLCN0HkkFqNjWdbJ0qRhLKkAgcrzzr9MmRCtUQn&amp;xkcb=SoAl67M2eDlWVygfKz0MbzkdCdPP&amp;fccid=29d37d43c382c8fe&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=52095026d7d936b1&amp;bb=ez91sI_i5AG6dZ3D-oMOPpVZfsJLfx6bvu6cbqQ1KTNZtdJ9W_iQ0Kxsvf_5UqYEjJbfKxzJB_QSoQlgCkLR440TLMVNPrPAelR8CzttM1iDg_uccdBPcrNNX0XF71g9&amp;xkcb=SoDM67M2eDlWVygfKz0DbzkdCdPP&amp;fccid=810178099fb1fcbc&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=074a3276d267f80a&amp;bb=ez91sI_i5AG6dZ3D-oMOPthx-XIzOuyB7-eln5u2B5dgridpTqzRoE4jwnUexNpKCV_0eGDIKaV3wA5OUZhKhP9Eo9X2jEEmZNz43XhZWQNLU2A05pQlDLy2dxoeQI4B&amp;xkcb=SoB467M2eDlWVygfKz0CbzkdCdPP&amp;fccid=b90433ed96d63887&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=8e2db73d56fb92c1&amp;bb=ez91sI_i5AG6dZ3D-oMOPngQLsROysTxWFrYV12QEm0CcCkaMfiIUNZXXit3WVM6Qr6ztyuogA3XvYazoWO2kHNDhf1tRsTKRruzdq3NvPeWKLa9cVtuELU9L6KDMoKo&amp;xkcb=SoDl67M2eDlWVygfKz0BbzkdCdPP&amp;fccid=fb92a252ae5b2ecc&amp;cmp=Technossus-Software-Services%2CChandigarh&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=e0c34264d46de58c&amp;bb=ez91sI_i5AG6dZ3D-oMOPhDDgQXkY9dbEnhSyk7p5xfTVh3CG0Dg8UwTjpoCuSyGBUXDm1h7PW9Lvn1BXQv8tgRtPE0uL7v__VXW1EOmdc7hqUU-NHDBdq6yC4HCbab9&amp;xkcb=SoBR67M2eDlWVygfKz0AbzkdCdPP&amp;fccid=3b98171e4a0fd997&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=e14addd0d99ff73d&amp;bb=ez91sI_i5AG6dZ3D-oMOPvhNhOYe-fVcXGEb8-DBnHatAP5-WO-BVqKeEVFv3rN3IwjBy7iywEJf8N63RJvsWoeS3DDraA9ofrgToDcI4zU7ZbAn_npvCU6t2aSBA4Th&amp;xkcb=SoDf67M2eDlWVygfKz0HbzkdCdPP&amp;fccid=659d7ed1b53f4cd4&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=93b6c468a9a12e86&amp;bb=ez91sI_i5AG6dZ3D-oMOPvQEY5dcgY8XTmckekBfOokZOqnVEQCRIgFbkjOed1FcB_B95-2i4YirAkAxn8h7-aME4eTHn3wxARQUTkpVQOJcMACUEzFVqjYu0YGLkrtn&amp;xkcb=SoBr67M2eDlWVygfKz0GbzkdCdPP&amp;fccid=74e36d81c894b4b7&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=456789abcdef0123</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=17a0927c427ef514&amp;bb=ez91sI_i5AG6dZ3D-oMOPh7o7V948syUNJG3LjkStVbXuZoeuEgrLgs92QPu1Vqtoe7BYOZiP7-nLfYzKBwRSmPlwX7EU9LaivqoFAdhaD-Zze3lEGt6GxRE4i0ADQtN&amp;xkcb=SoD267M2eDlWVygfKz0FbzkdCdPP&amp;fccid=dd616958bd9ddc12&amp;cmp=Zentrumhub-Solutions&amp;ti=Senior+.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Synextic Global Business Solution</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>3-5 years</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-synextic-global-business-solution-JV_KO0,13_KE14,47.htm?jl=1009542027944</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>

</xml_diff>

<commit_message>
Update job search descriptions and default experience selection in index.html
- Changed subtitle to reflect searching across all configured portals.
- Updated default experience selection from "3-5 years" to "5-8 years".
- Revised footer text to clarify that searches include all URLs listed in jobs_input.xlsx.
</commit_message>
<xml_diff>
--- a/scraped_jobs_permanent.xlsx
+++ b/scraped_jobs_permanent.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,22 +461,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>.NET Full Stack Developer with Angular</t>
+          <t>Junior .Net developer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Verveba Telecom</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-with-angular-verveba-telecom-JV_IC2856202_KO0,37_KE38,53.htm?jl=1010253578252</t>
+          <t>https://in.linkedin.com/jobs/view/junior-net-developer-at-sonata-software-4477830244</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -503,22 +503,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>.NET Full Stack Developer</t>
+          <t>Senior .NET Developer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TMC Pvt Ltd</t>
+          <t>P99SOFT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-tmc-pvt-ltd-JV_IC2940587_KO0,24_KE25,36.htm?jl=1010289170116</t>
+          <t>https://in.linkedin.com/jobs/view/senior-net-developer-at-p99soft-4477575431</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -545,22 +545,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>.NET Full Stack Developer</t>
+          <t>Professional Full Stack .NET Developer (F/M/D)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Carvewing</t>
+          <t>Freudenberg Filtration Technologies</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-carvewing-JV_IC2940587_KO0,24_KE25,34.htm?jl=1007577157324</t>
+          <t>https://in.linkedin.com/jobs/view/professional-full-stack-net-developer-f-m-d-at-freudenberg-filtration-technologies-4471869237</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -592,17 +592,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>.Net Full Stack Developer</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MetaDesign Solutions</t>
+          <t>Luxoft</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gurgaon</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-metadesign-solutions-JV_IC2921225_KO0,24_KE25,45.htm?jl=1010285486155</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-luxoft-JV_IC2856202_KO0,13_KE14,20.htm?jl=1010288217956</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,22 +629,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.NET Developer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>MHTECHIN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=d9afc88f5c049c6d&amp;bb=YKSahP_QOR2BrlEPW1bY-pNTHC1apHWfYwpaAorXXcfbRYG6oVqcQ3but_8oUutFJyW5sLncUbwbcT3i5cIgsHziJGT0_s3Sy5SqC6MUYWuizUuQQ5MMNYKJ6cSLIMhq&amp;xkcb=SoBE67M2d0QpkET7jx0LbzkdCdPP&amp;fccid=1f5c7702a1640572&amp;cmp=Steerlean-Consultancy-Services-Pvt.-Ltd.&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-mhtechin-JV_IC2856202_KO0,13_KE14,22.htm?jl=1010195050015</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -671,22 +671,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net developer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Elysiar Technologies</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=8da132067a94c560&amp;bb=YKSahP_QOR2BrlEPW1bY-j2I3WCOkd8Fp9nHf40gU9m9DCgbBnGCVAb6Tyy_ZKGoNbWSjGDynLFSYkFSR84DQ7RcAbk_A-nfin24XId7gybLNNftdeC0w1ZZ0LXG1Jsn&amp;xkcb=SoDw67M2d0QpkET7jx0KbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-elysiar-technologies-JV_IC2856202_KO0,13_KE14,34.htm?jl=1006887054899</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -713,22 +713,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>C#.Net Developer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=5e65a788077721ca&amp;bb=YKSahP_QOR2BrlEPW1bY-ir81OGfYg3jXWf395rxzh9_MAdtkFXuehHDVG74yhZ5hP5-zS5ZMPKe6rT0G4_zqwNY5sMkGt_il_q63lTiQHresruOwPrNBLaEo0amZT2_&amp;xkcb=SoBt67M2d0QpkET7jx0JbzkdCdPP&amp;fccid=ea6bb53f0b18b8f2&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/c-net-developer-wipro-JV_IC2856202_KO0,15_KE16,21.htm?jl=1010297859203</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -755,22 +755,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.NET Developer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Siddhatech Software Services</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=807e439b26cfd6ac&amp;bb=YKSahP_QOR2BrlEPW1bY-n8kbci8poWDGgHv6vIh0ew4UuLT25y58sf0wbpqWDQa2LOW9-cYAlCNigDUmeBc4M3xtEmsA-qKAG5bvwI50yw1M085TAkD_6hTfRhLmNEU&amp;xkcb=SoAB67M2d0QpkEz7jx0LbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-siddhatech-software-services-JV_IC2856202_KO0,13_KE14,42.htm?jl=1005897504638</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -797,22 +797,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>IT Shastra</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -822,7 +822,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=766ea748f5354651&amp;bb=YKSahP_QOR2BrlEPW1bY-ir81OGfYg3jmOw7b2Kgxm4NJp1sP-MRqJRbqn9x09Y1cDBlt_N_ty5hgACgqNYfSdfpXNq-wrWjF6zfmnrcWgx4lZ284gQ4QPR38E-7gjoO&amp;xkcb=SoC167M2d0QpkEz7jx0KbzkdCdPP&amp;fccid=99b9b1212188b67d&amp;cmp=Rosemallow-technologies&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-it-shastra-JV_IC2856202_KO0,13_KE14,24.htm?jl=1010106159756</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -839,22 +839,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer, AS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Deutsche Bank</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=b0d00ff6f2716b68&amp;bb=YKSahP_QOR2BrlEPW1bY-nypeiEkCXmFA4ctiZBTkKC1WfOIjL1S3dpxtV-c3nVp61z_TTW25RishZdOG3D4FoZ25qduxkTqH3oMFPm6dvHwhzsV25tWhNLT9zKLKX_G&amp;xkcb=SoAo67M2d0QpkEz7jx0JbzkdCdPP&amp;fccid=c5679bf29a1db253&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-as-deutsche-bank-JV_IC2856202_KO0,16_KE17,30.htm?jl=1010088302927</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -881,22 +881,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Swipfe Infotech</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=218f0f4a6447640b&amp;bb=YKSahP_QOR2BrlEPW1bY-qiq6eMtvk2PMA8_AStoIRtbOix-Dl5v2erioTMWRv2FC_UEIlYjFILgbEzzaPOyhdTjq9KCnpNNGUw_q8_8-_w6FMNjw_tUhz5w4-Sv3IYx&amp;xkcb=SoCc67M2d0QpkEz7jx0IbzkdCdPP&amp;fccid=15f3dea53ebe3c30&amp;cmp=Countless-services-private-limited&amp;ti=.NET+Developer&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-swipfe-infotech-JV_IC2856202_KO0,13_KE14,29.htm?jl=1009972384828</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -923,22 +923,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Bio-Analytical Technologies</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=799784c7fd9c5c05&amp;bb=YKSahP_QOR2BrlEPW1bY-qrNAiE5DtEzVGNv67h0ac9-K5P6mxqxMbOF9qYeUQnjoDRFowDO-Bs1EvzDtppkcjugJVadw8CRGxrA4jTsfrxm43tEET011062WcVCCVlV&amp;xkcb=SoAS67M2d0QpkEz7jx0PbzkdCdPP&amp;fccid=2fad1b49105da4f2&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-bio-analytical-technologies-JV_IC2856202_KO0,13_KE14,41.htm?jl=1005721998145</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -965,22 +965,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Lead .Net Developer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Komax Group</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=e87d802dead8432d&amp;bb=YKSahP_QOR2BrlEPW1bY-qudCTHZP3BnHlNk3hsx3ChKabkJdcnOh6bAYFRB-HTSsDSvJp0ofL0whsEv32DD4cP8X_qk9JTu3luqV61p9NLTldyEZYIhwdUL89K0-EjX&amp;xkcb=SoCm67M2d0QpkEz7jx0ObzkdCdPP&amp;fccid=2fad1b49105da4f2&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/lead-net-developer-komax-group-JV_IC2856202_KO0,18_KE19,30.htm?jl=1010296980923</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1007,22 +1007,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>VB.NET Developer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Rosemallow Technologies</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=52d1b74ff1a5d229&amp;bb=YKSahP_QOR2BrlEPW1bY-pBwA0tNns7IdpdlPxYKOIDxedP6BKooRbYf4_8ymLkazJWQNbkmHpDPVZBnGlU7ceAKK7zh4qq55rUY0Oz6KG1c26JT-TDwDO95Li__TtHB&amp;xkcb=SoA767M2d0QpkEz7jx0NbzkdCdPP&amp;fccid=0d1386ca25efa609&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/vb-net-developer-rosemallow-technologies-JV_IC2856202_KO0,16_KE17,40.htm?jl=1010292479919</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1049,22 +1049,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Mechatronics Systems</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=79e3a0117be104c0&amp;bb=YKSahP_QOR2BrlEPW1bY-rpxjdquZm9ouDy05Uk8S83azceN5JuFAJ4Mu-zBpbGqWMV8IjCOvzyaoKRYAAVbd9FImYTfeKbBOAq9he8oQrKjWTIsSEtzcn7VVsREaPIJ&amp;xkcb=SoCP67M2d0QpkEz7jx0MbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-mechatronics-systems-JV_IC2856202_KO0,13_KE14,34.htm?jl=1008234944903</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1091,22 +1091,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Professional Full Stack .NET Developer (F/M/D)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Freudenberg Group</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=467ae9c642e93e56&amp;bb=YKSahP_QOR2BrlEPW1bY-pWHDuKxNxrh4CrCnmo3yzSDYdN1ajygb72k2T1pwhbvxAylWUTSX40gRqhy4x71ukKvAJBlJx49jk7OUB8SML1OhcPFHRcxMyl7urExyUab&amp;xkcb=SoBm67M2d0QpkEz7jx0DbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/professional-full-stack-net-developer-fmd-freudenberg-group-JV_IC2856202_KO0,41_KE42,59.htm?jl=1010286977718</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1133,22 +1133,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Asp .Net Developer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Vision Cloud</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/viewjob?jk=a1b2c3d4e5f67890</t>
+          <t>https://www.glassdoor.co.in/job-listing/asp-net-developer-vision-cloud-JV_IC2856202_KO0,17_KE18,30.htm?jl=1007660714907</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1175,22 +1175,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Triotech Software System</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=42e34127a672abcf&amp;bb=YKSahP_QOR2BrlEPW1bY-pFdrhCSNmmVXs5k0ViQRQBPoxLWLEIdLcgTqx9nZbk6Xc8zUuh9H637nRu5831lE35qO31KCdOOGAO8vkJQyLxraQqujM5LAjaynrjYZeQE&amp;xkcb=SoDS67M2d0QpkEz7jx0CbzkdCdPP&amp;fccid=1174e11d97fd620e&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-triotech-software-system-JV_IC2856202_KO0,13_KE14,38.htm?jl=1007872878984</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1217,22 +1217,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Aarohiinfo FI Management</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=95a4ff7430f1548d&amp;bb=YKSahP_QOR2BrlEPW1bY-l6aqphC702ta3SP7vof5n73WBBoNlLam7xc0feKl2BnY5pFV7_9rZuPJBOUNhKVM2sxM3v4Oc327AlemUIatxpe84LqFeC05cWb7Fy_xOoE&amp;xkcb=SoBP67M2d0QpkEz7jx0BbzkdCdPP&amp;fccid=91444a28cb181211&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-aarohiinfo-fi-management-JV_IC2856202_KO0,13_KE14,38.htm?jl=1008913612152</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1259,22 +1259,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Proventeq</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://in.indeed.com/rc/clk?jk=2aa74008fc68d77c&amp;bb=YKSahP_QOR2BrlEPW1bY-tJQhkc9oJgfnUb7ykUnSym19GsWOV87-mOddMXVK7vP3n24YY2XpGtnanS4TFSexmC6fsdFrISn-6i_TqMUz--9SO5FuC51QbjFW31_h5SX&amp;xkcb=SoD767M2d0QpkEz7jx0AbzkdCdPP&amp;fccid=b90433ed96d63887&amp;vjs=3</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-proventeq-JV_IC2856202_KO0,13_KE14,23.htm?jl=1008311011631</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>.Net Full Stack Developer</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Truviq Systems</t>
+          <t>MDI NetworX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Hyderābād</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-truviq-systems-JV_IC2865319_KO0,24_KE25,39.htm?jl=1010297997067</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-mdi-networx-JV_IC2856202_KO0,13_KE14,25.htm?jl=1010065634540</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1348,17 +1348,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Senior .NET Full Stack Developer</t>
+          <t>.Net Developers</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eins Technology</t>
+          <t>Salus Technologies</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/senior-net-full-stack-developer-eins-technology-JV_KO0,31_KE32,47.htm?jl=1010205531106</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developers-salus-technologies-JV_IC2856202_KO0,14_KE15,33.htm?jl=1006549799469</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1385,22 +1385,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>.NET Full Stack Developer</t>
+          <t>Senior .Net Developer8 - 15 yrsPune443+ ReviewsC#.Net.Net CoreEntity FrameworkPosted 1 week agoPosted 1 week ago</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Cyber Infrastructure (CIS)</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Indore</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-cyber-infrastructure-cis-JV_IC2876676_KO0,24_KE25,49.htm?jl=1010302372870</t>
+          <t>https://www.hirist.tech/j/senior-net-developer-1678746?ref=sp&amp;jobPos=2</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1427,22 +1427,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>.NET Full Stack Developer</t>
+          <t>.Net Developer5 - 8 yrsGurgaon/Gurugram.NetC#.Net CoreOOPSEntity FrameworkPosted 1 month agoPosted 1 month ago</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hyderābād</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-persistent-systems-JV_IC2865319_KO0,24_KE25,43.htm?jl=1010272991493</t>
+          <t>https://www.hirist.tech/j/net-developer-1673958?ref=sp&amp;jobPos=3</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1469,40 +1469,1552 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>.Net Developer - C#/ASP5 - 9 yrsHyderabad3.991+ Reviews.NetASPMultithreadingC#Posted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-asp-1674099?ref=sp&amp;jobPos=5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>.Net Developer4 - 6 yrs10-15 LPAGurgaon/Gurugram.NetC#.Net CoreSQL ServerASPPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-1671544?ref=sp&amp;jobPos=6</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>.Net Developer - Distributed Backend4 - 6 yrsBangalore.NetC#ASPPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-distributed-backend-1672423?ref=sp&amp;jobPos=7</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Senior .Net Developer - Banking/Insurance Domain5 - 10 yrsMultiple Locations.NetC#Data StructureAlgorithmPosted 2 weeks agoPosted 2 weeks ago</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/senior-net-developer-banking-insurance-domain-1677649?ref=sp&amp;jobPos=9</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>.Net Developer - ASP/C#4 - 6 yrsGurgaon/Gurugram.Net.Net CoreC#SQL ServerPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-asp-c-1671638?ref=sp&amp;jobPos=11</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>.Net Developer - C# Programming8 - 20 yrs20-25 LPAMultiple LocationsMay work from homeC#.NetSDLCSystem DesignPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-programming-1671136?ref=sp&amp;jobPos=12</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>.Net Developer - C#/AngularJS5 - 8 yrsBangalore.Net.Net CoreAngularJSSQL ServerC#ASPTypeScriptFull Stack+3Posted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-angularjs-1670525?ref=sp&amp;jobPos=15</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>.Net Developer - C#/WPF5 - 8 yrsBangalore.Net.Net CoreC#WPFMultithreadingC+++1Posted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-c-wpf-1670227?ref=sp&amp;jobPos=16</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>.Net Developer5 - 7 yrsMumbai.Net.Net CoreC#ASPPosted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-1667585?ref=sp&amp;jobPos=17</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>.Net Developer - ASP/MVC5 - 10 yrsBangalore4.324+ Reviews.NetBackend ArchitectureASPMVC.Net CoreC#+1Posted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/net-developer-asp-mvc-1669727?ref=sp&amp;jobPos=18</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Senior .Net Developer - C#/React.js8 - 12 yrsBangaloreC#.NetOpenAI.Net CoreReact.jsAngularJSFull Stack+2Posted 1 month agoPosted 1 month ago</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>www.hirist.tech</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/senior-net-developer-c-reactjs-1673568?ref=sp&amp;jobPos=20</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>.Net developer jobs pune indiawork from home</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntr3hdahkGMqLucgtY6Jy5syj3Vfw:1792763564023&amp;q=.Net+developer+jobs+pune+india+work+from+home&amp;sa=X&amp;ved=2ahUKEwjPg5nbpNCXAxWrPDQIHeCdOQoQ1QJ6BAhQEAE</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>.Net developer jobs pune indiasalary</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntr3hdahkGMqLucgtY6Jy5syj3Vfw:1792763564023&amp;q=.Net+developer+jobs+pune+india+salary&amp;sa=X&amp;ved=2ahUKEwjPg5nbpNCXAxWrPDQIHeCdOQoQ1QJ6BAhFEAE</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>.Net developer jobs pune indiafor freshers</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntr3hdahkGMqLucgtY6Jy5syj3Vfw:1792763564023&amp;q=.Net+developer+jobs+pune+india+for+freshers&amp;sa=X&amp;ved=2ahUKEwjPg5nbpNCXAxWrPDQIHeCdOQoQ1QJ6BAhBEAE</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Remote .NET developer Jobs (October 2026) - Arcarc.devhttps://arc.dev› Remote Jobs</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.google.com/goto?url=CAESXgHrOzAVCbvde7V6bcZamEnbtfGUTuWAq99dQ_R8mdXC928nv6yN-wrMH1bu01miGwU4GmiNJwl2z80pIeFtolO2raDITZO6uqe2EauJ6ceDs7B9PZEssNlVK1GC06k</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Remote .NET Developer Jobs in 2027Wellfoundhttps://wellfound.com› role › .net-developer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.google.com/goto?url=CAESZgHrOzAVyc8HMJN3MWSlKIZslHsGeBbspMXA79hCfo3IdIorL9CaNt-i5R-8yJbiTzDzvQoNHhH3PLxTH7f_WVTNsEwgVRaShST2mnulfJiqc8I-oyLDJzXgUFQTPKXA1O6_0G-SCA</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>.Net developer jobs remoteindia</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+india&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhLEAE</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>.Net developer jobs remoteworldwide</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+worldwide&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhiEAE</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>.Net developer jobs remotesalary</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+salary&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhlEAE</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>.Net developer jobs remotepart time</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>www.google.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+part+time&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhmEAE</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=8da132067a94c560&amp;bb=Hcx10gWOKryWGOh2y_7EE5QpFoqHsQNuAuapk5HKINXEnKcTUmVFaXzvbQvxrEBRoVYmPzjYtQu4LQfDtMK-RX-wd96d1rg33Twkql-aMnhs3Rp-VB7jBsEL9jBg_dlZ&amp;xkcb=SoCa67M2d0pPouz4BJ0LbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=006a32d5fe51635c&amp;bb=Hcx10gWOKryWGOh2y_7EE-Q8MMWd47rzMJebH_pyGCgl25D2AG3yEYhtEzy_fKCuMJ-uT7MdXCghLWgIh4bQ2r8BN9gy7egXBE5NRJeq5AbiYUysj7Ims9AcEdG81-48&amp;xkcb=SoAu67M2d0pPouz4BJ0KbzkdCdPP&amp;fccid=3d3123a1ac04ce14&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=766ea748f5354651&amp;bb=Hcx10gWOKryWGOh2y_7EE33U3WPWSpyth_0atSPz4CoA6hKMgDIJ4uQuzvJRiXRX9YwQsz3x6b6r8fwHZ3FhY0y1-Hg2OFjIn30MG-IeFNOdCzBrVuGBaFayv9Cxh1d3&amp;xkcb=SoCz67M2d0pPouz4BJ0JbzkdCdPP&amp;fccid=99b9b1212188b67d&amp;cmp=Rosemallow-technologies&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=f04131cb17a8aa32&amp;bb=Hcx10gWOKryWGOh2y_7EE5vvfVvz3QB7f1yBYqIiMzHnyMGgVbdj8OVT84YYsdrmYutgCYqSGsPBmhfbl5BEFRuTZYgRwwd8kQTeFh2Sv5qZqDagoiij9rSgFGazPMKe&amp;xkcb=SoAH67M2d0pPouz4BJ0IbzkdCdPP&amp;fccid=7a162ca462563282&amp;cmp=Senwell-Solutions&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=d9afc88f5c049c6d&amp;bb=Hcx10gWOKryWGOh2y_7EE-rPlnHqhTOkkEH3_Mt9T34F3rY0AcavGqyGocIVQlisQGdJTy3IIUxYGOR5yFYj6DCeFktPR8tgnpB_Q0ArATrQV909VPuf_8JEHIv9cQeA&amp;xkcb=SoCJ67M2d0pPouz4BJ0PbzkdCdPP&amp;fccid=1f5c7702a1640572&amp;cmp=Steerlean-Consultancy-Services-Pvt.-Ltd.&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=218f0f4a6447640b&amp;bb=Hcx10gWOKryWGOh2y_7EE3ChwAOoQd1Apv_Tssmn-8clmxgZXb-nw5fye9jpEhNm5gj1GVEA3H4iev9qBb6dye9a_SAgGyBBGYZO_BCLf7j39T8xV_DBHv4iFBBdT-Ui&amp;xkcb=SoA967M2d0pPouz4BJ0ObzkdCdPP&amp;fccid=15f3dea53ebe3c30&amp;cmp=Countless-services-private-limited&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=566bdc09a50bcd32&amp;bb=Hcx10gWOKryWGOh2y_7EE7lXIprlQrgW94vy17jdL0rjrqS0gyZhQUksZnmPUMq3neQBzllr0C08pm1A2lvu-6Y4r72YXhbC3l538Z7To6RyNn0g0SlZ3pxmysVNxBVO&amp;xkcb=SoCg67M2d0pPouz4BJ0NbzkdCdPP&amp;fccid=c3d73a6fd53e8543&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=1782c21af7e0df75&amp;bb=Hcx10gWOKryWGOh2y_7EE6FqiodHdkZehui-OyBUzcr4L82Th7_uuIMDXloyiJNtCEvO7i8n_l6FsU2OFASDGY_5hUEmCoGhYKCctLi0Ng-qYnl7JQ9Fs9drFO4Siity&amp;xkcb=SoAU67M2d0pPouz4BJ0MbzkdCdPP&amp;fccid=74e36d81c894b4b7&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=f6f2cf53a58a0fad&amp;bb=Hcx10gWOKryWGOh2y_7EE8eB_y_GBR24v-O0QJ7AlMWIK_vn1XgBk5LzOcgPLpSVzhst_I6baR4GW0jme5dEiKtiyZU32Z-pPRLGbhUKmE0W6qOxNUsGBmaRoMQ7Jo0p&amp;xkcb=SoD967M2d0pPouz4BJ0DbzkdCdPP&amp;fccid=464e2ee7fbea2edc&amp;cmp=SphereGen-Technologies&amp;ti=Senior+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=79e3a0117be104c0&amp;bb=Hcx10gWOKryWGOh2y_7EE5qFmL_xhzR1S3W6gmsAapVCd0gLlN8gIewNczww7wyqtN2Rlv45PS4NSKOlb40aSXq5yr5zIyXZ7dAM_FrMZwBFGv0qTGXJDJwMtQY8hyPS&amp;xkcb=SoBJ67M2d0pPouz4BJ0CbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=807e439b26cfd6ac&amp;bb=Hcx10gWOKryWGOh2y_7EE-uwu6I-hyrCsvwTNvhgXkOyb7jbpJw_xiI3QKJvsC7n1Asc3GT7ijAuKUsO4RchwkkKxNPYbV8B-3KdY99neorIfc-7OFj3k7I7tyM6RFE2&amp;xkcb=SoDU67M2d0pPouz4BJ0BbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=e87d802dead8432d&amp;bb=Hcx10gWOKryWGOh2y_7EE4rbgza9sJw-7z94nnZKfNakGTsb-0TYL_edkDm2AXIfDKHh4vnMqk_hL41NNnefjbU3AsYK_Y7-dKDYRVx45yJxvlSnbTEs92X9OvzMFp1o&amp;xkcb=SoBg67M2d0pPouz4BJ0AbzkdCdPP&amp;fccid=2fad1b49105da4f2&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=df1aa1127172a51f&amp;bb=Hcx10gWOKryWGOh2y_7EE-uwu6I-hyrCTFaHZ3myIXZTIrLK3VrlVPqPmqFF628DY7z4p9mwpRRXwTRmAOVx8Kd5tAzKbORRIPCLgGjvjakyaYPYIZpf_bhUpUU9G0eJ&amp;xkcb=SoDu67M2d0pPouz4BJ0HbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=2aa74008fc68d77c&amp;bb=Hcx10gWOKryWGOh2y_7EE1W7ljh1w4ER_EHxQg9LUDnU39S6q_zDyFM9qkEuVWBJH__NCdnBj_n0q5Ow1HrS493eYeqmeN7CQETpmOisW7fEkW55Eb60mbWQSPgmLLlh&amp;xkcb=SoBa67M2d0pPouz4BJ0GbzkdCdPP&amp;fccid=b90433ed96d63887&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=cdef0123456789ab</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=b212ad1b8a056e3a&amp;bb=Hcx10gWOKryWGOh2y_7EEwK02jMB57x59l-xgPHPMV2drIXGa2bp3gJ5CJHFYHsOPr41bBcMHd0QQubsVlb5zoeMefIduFhDtS8X9yQzo6EDlXyXV8pVvBv-zfZYwrTI&amp;xkcb=SoDH67M2d0pPouz4BJ0FbzkdCdPP&amp;fccid=105ecfd0283f415f&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>Glassdoor</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>.Net Full Stack Developer</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>E-Merge tech</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>5-8 years</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-full-stack-developer-e-merge-tech-JV_IC2833209_KO0,24_KE25,37.htm?jl=1009492088180</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Refer to Apply Link</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>.Net Developer</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Realizer Technologies</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-realizer-technologies-JV_KO0,13_KE14,35.htm?jl=1007531044310</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>

</xml_diff>

<commit_message>
fix: update table header to include 'Posted' column for better clarity
</commit_message>
<xml_diff>
--- a/scraped_jobs_permanent.xlsx
+++ b/scraped_jobs_permanent.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,15 +444,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Posted Age Days</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Apply Link</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Recruiter Contact</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Job Type</t>
         </is>
@@ -466,12 +471,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Junior .Net developer</t>
+          <t>Senior .NET Developer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>P99SOFT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -484,17 +489,20 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/junior-net-developer-at-sonata-software-4477830244</t>
-        </is>
+      <c r="F2" t="n">
+        <v>11.63556069435185</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.linkedin.com/jobs/view/senior-net-developer-at-p99soft-4477575431</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -508,12 +516,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Senior .NET Developer</t>
+          <t>Professional Full Stack .NET Developer (F/M/D)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P99SOFT</t>
+          <t>Freudenberg Filtration Technologies</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -526,17 +534,20 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-net-developer-at-p99soft-4477575431</t>
-        </is>
+      <c r="F3" t="n">
+        <v>7.635560708715277</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.linkedin.com/jobs/view/professional-full-stack-net-developer-f-m-d-at-freudenberg-filtration-technologies-4471869237</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -545,22 +556,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Professional Full Stack .NET Developer (F/M/D)</t>
+          <t>VB.NET Developer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Freudenberg Filtration Technologies</t>
+          <t>Rosemallow Technologies</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -568,17 +579,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/professional-full-stack-net-developer-f-m-d-at-freudenberg-filtration-technologies-4471869237</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/vb-net-developer-rosemallow-technologies-JV_IC2856202_KO0,16_KE17,40.htm?jl=1010292479919</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -592,12 +604,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>Lead .Net Developer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Luxoft</t>
+          <t>Komax Group</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -610,17 +622,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-luxoft-JV_IC2856202_KO0,13_KE14,20.htm?jl=1010288217956</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/lead-net-developer-komax-group-JV_IC2856202_KO0,18_KE19,30.htm?jl=1010296980923</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -634,12 +647,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>.NET Developer</t>
+          <t>.Net Developer, AS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MHTECHIN</t>
+          <t>Deutsche Bank</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -652,17 +665,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-mhtechin-JV_IC2856202_KO0,13_KE14,22.htm?jl=1010195050015</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-as-deutsche-bank-JV_IC2856202_KO0,16_KE17,30.htm?jl=1010088302927</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -671,22 +685,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>www.placementindia.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>.Net developer</t>
+          <t>Apply to 109 .Net Developer Job Vacancies in Pune</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Elysiar Technologies</t>
+          <t>www.placementindia.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -694,17 +708,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-elysiar-technologies-JV_IC2856202_KO0,13_KE14,34.htm?jl=1006887054899</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.placementindia.com/job-search/full-stack-web-developer-jobs-in-pune.htm</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -713,22 +728,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C#.Net Developer</t>
+          <t>Senior .Net Developer8 - 15 yrsPune443+ ReviewsC#.Net.Net CoreEntity FrameworkPosted 1 week agoPosted 1 week ago</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -736,17 +751,20 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/c-net-developer-wipro-JV_IC2856202_KO0,15_KE16,21.htm?jl=1010297859203</t>
-        </is>
+      <c r="F8" t="n">
+        <v>7</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.hirist.tech/j/senior-net-developer-1678746?ref=sp&amp;jobPos=2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -755,22 +773,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>.NET Developer</t>
+          <t>Senior .Net Developer - Banking/Insurance Domain5 - 10 yrsMultiple Locations.NetC#Data StructureAlgorithmPosted 2 weeks agoPosted 2 weeks ago</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Siddhatech Software Services</t>
+          <t>www.hirist.tech</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -778,17 +796,20 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-siddhatech-software-services-JV_IC2856202_KO0,13_KE14,42.htm?jl=1005897504638</t>
-        </is>
+      <c r="F9" t="n">
+        <v>14</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.hirist.tech/j/senior-net-developer-banking-insurance-domain-1677649?ref=sp&amp;jobPos=9</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -797,22 +818,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>Dot Net Developer Jobs In Pune</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>IT Shastra</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -820,17 +841,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-it-shastra-JV_IC2856202_KO0,13_KE14,24.htm?jl=1010106159756</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScAHrOzAV5fIeL0_Wek5NV7joSGViyH4UweWw_Mv2MWAAIiQM-E6kMye_R5XkoLABt49Ba0p3viFk5OP4MTRrEQ6EKgTrJ7hyWwBu45kcocrU7ycIgey-6S5UL-X4o0r69dSllos5uC1sTKpUC5uDFkk</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -839,22 +861,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>.Net Developer, AS</t>
+          <t>Dotnet Developer Jobs in Pune (1000+ Open Roles)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Deutsche Bank</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -862,17 +884,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-as-deutsche-bank-JV_IC2856202_KO0,16_KE17,30.htm?jl=1010088302927</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScgHrOzAV2hiyM9xWguSbWwdxB68N_m3gXauubti07cxuFS2HdWh83CtU6sN1z-vfiMf6hV9533P-TF4LxX2EEk3OWRD38t8Cv1plND4QoyLxYgeOi9zrHnYfzLRnr-zEmCZBVm5F4aPgEyHpBmMFJPmCyQ</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -881,22 +904,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>400 Net Developer Job Vacancies in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Swipfe Infotech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -904,17 +927,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-swipfe-infotech-JV_IC2856202_KO0,13_KE14,29.htm?jl=1009972384828</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESfgHrOzAVjyLZggOxbDej49drhpLjTBYDcZv44pGH8QwWWWnrsBjmA1Gs_9_CUQrehsNJnajDftNZ3ZU2NrgJOIhwDH2FYqzobE7sx4lAt9ESp-f2njodjTRCdwZxMaiIWaHTGg2ooI5yxfkPvtm-yWjTmK4TbY6q5musf33IMQ</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -923,22 +947,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>DOT NET Developer Jobs in Pune</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bio-Analytical Technologies</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -946,17 +970,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-bio-analytical-technologies-JV_IC2856202_KO0,13_KE14,41.htm?jl=1005721998145</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESgQEB6zswFfPZXzybGyWv9_KvGtpHhxN7fcMjySOTT_gTH7HeUw8vtS1l3mvcsv8FagdugqfY1DKgF38CntkeLXrLJDOSYiOS9qWeTRoNZ0M_fi8UE-cudMfkRE-8dB9Zq5YTFuPtT6je__-CrY04f3KonFp2VUITbM6ges6YvRPHHTA</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -965,22 +990,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lead .Net Developer</t>
+          <t>Best NET Developer Jobs in Pune 2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Komax Group</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -988,17 +1013,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/lead-net-developer-komax-group-JV_IC2856202_KO0,18_KE19,30.htm?jl=1010296980923</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESewHrOzAVRNl44XIdYMkyUc8RH6_GWWyDR_MHxtthrPj8GMnRcKQbMJshgq9osLkcvjwpAJTB6XlTFzX_i3ZdSflfcatDoqGULjFMa3BC0aVU6ztOa5pGPuidLYURyLhPElj3WQv3ylDJCICIem14pnkxCffPclAV9tScpw</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1007,22 +1033,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VB.NET Developer</t>
+          <t>152+ .Net Jobs in Pune | .Net Job openings in Pune</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rosemallow Technologies</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1030,17 +1056,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/vb-net-developer-rosemallow-technologies-JV_IC2856202_KO0,16_KE17,40.htm?jl=1010292479919</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZwHrOzAVe9GAxNaAPpUD80FRTC9TxZHWHspY9yX6vRhwucIpXzDYXodoacf1CiGhVserD-21DkoTdnKeYcPg0CBnZhq0wd8PP4bIdXmLvd3E7xzUVyBeEkJ0cpfb4P0HlyCXXv6VqrU</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1049,22 +1076,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>1691 Dotnet Job Vacancies In Pune</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mechatronics Systems</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1072,17 +1099,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-mechatronics-systems-JV_IC2856202_KO0,13_KE14,34.htm?jl=1008234944903</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZQHrOzAV-43z0gyyB5Pk8zwy9vbYbcPyd52vdhjuVLyGifFw02VxvL2Dhlse7gxa1e7Wyt3cp_uewIiCenEoKnxtsFXqGbFzamCQ5hG2N53JcqcskHY09lgh408h6sDjEn3C3CPm</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1091,22 +1119,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Professional Full Stack .NET Developer (F/M/D)</t>
+          <t>382 pune net developer Jobs in India, August 2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Freudenberg Group</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1114,17 +1142,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/professional-full-stack-net-developer-fmd-freudenberg-group-JV_IC2856202_KO0,41_KE42,59.htm?jl=1010286977718</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEShgEB6zswFUvu28_3fwg8R7qB_bmIgbcAFif6NAlhTCWXJERIFL_-5NaLgZz_u4xWmnjoS_dGyMnoitv1DbpSkXFSSYnNVX9EgQzGO-8W7tWkdigOd8DMBT18nDB-rlBRhN_7ngaVHTMwaGV2jtYH_dceCzwCROq4xSbBifx383TWSOxsZ11iZQ</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1133,22 +1162,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Asp .Net Developer</t>
+          <t>Dot Net Developer Jobs In Pune</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vision Cloud</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1156,17 +1185,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/asp-net-developer-vision-cloud-JV_IC2856202_KO0,17_KE18,30.htm?jl=1007660714907</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScAHrOzAVdhLH0DMZHFoZrc7a61eCVaJTy8xmT1FXQiV7wSHsvxNwJXn4ynIBKoTNKi-Z-t406RyYJAJAWd8kjHfDJCkZdTqBbNHaowLtF1EYXEGsQuuenH2tDqRLzIGfqp7X5yS4Azte_HAtzJTo_Z8</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1175,22 +1205,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>Dotnet Developer Jobs in Pune (1000+ Open Roles)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Triotech Software System</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1198,17 +1228,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-triotech-software-system-JV_IC2856202_KO0,13_KE14,38.htm?jl=1007872878984</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScgHrOzAVUA2N3j2jalYxlOIwSIj-24RytFWUx3FLeWwLSElDDmi60v2sZ-rHKZ3h0Q4Z9DO6nQI1paXa7VST42uBKVTE1zqLJTIG8PcsVW1G7hx57mYpkOFS7iSKNgheTWfrcNtfmUtPcpN-LOCx2B5h2A</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1217,22 +1248,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>400 Net Developer Job Vacancies in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Aarohiinfo FI Management</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1240,17 +1271,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-aarohiinfo-fi-management-JV_IC2856202_KO0,13_KE14,38.htm?jl=1008913612152</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESfgHrOzAVzvzAoktYt0iV6pSRm6s5slbVmmY_YzlpKLvMH26nlyJL_d0Axukv0j2AchAzvhcvjC-9prhqoVmIk0vQygpBoUrImzoWNtvzBErTJrPlm7NqPZtVwVezreedYL-fldqy_t_g2k8N250Kkk3Evzrzr2vXoTg2R-Znlg</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1259,22 +1291,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>DOT NET Developer Jobs in Pune</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Proventeq</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1282,17 +1314,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-proventeq-JV_IC2856202_KO0,13_KE14,23.htm?jl=1008311011631</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESgQEB6zswFRPQOinETrx4pMZ0Ns7Fr2SeTyxwz8xnKd0l-fcHGpvqiSC2CXysDSS_sSYyoZZM0AxkHNRj1F8lEfaJSSL13D4xevqEkqFh1v-wgUj7uqXidOVvZ8-zQeek-sOA7d1SQQNjswu2J-zF_lpJKAyEsR5f3M00Wss48li8LFQ</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1301,22 +1334,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>.Net Developer</t>
+          <t>Best NET Developer Jobs in Pune 2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MDI NetworX</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1324,17 +1357,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-mdi-networx-JV_IC2856202_KO0,13_KE14,25.htm?jl=1010065634540</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESewHrOzAVVcGX6ZioPDqrdzKQVMdPlqICRp-bUKHBiLN6gtMyheVSBxK7LUhTtLOtj7CghumeMoRCM2fXjhWvZl8DbWU72WtLJVa6e5srgxzPJpgDlOJvT7IuIGfdkFwVg-0QL8uSWmBVfl9m60-wsPWGqarvLH9xCXKu0A</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1343,22 +1377,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>.Net Developers</t>
+          <t>152+ .Net Jobs in Pune | .Net Job openings in Pune</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Salus Technologies</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1366,17 +1400,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developers-salus-technologies-JV_IC2856202_KO0,14_KE15,33.htm?jl=1006549799469</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZwHrOzAV-awwsmmuS6F0biqZgX6M6B63JblP9QhC3f58jQFtxrHHU-8GjXWJ_4r4Af4o5gZypL8wOeK3kLh1_Hf4QJorEe1PF2Jvyqgnjx1Z4GqGKpCNww-lyqsOssbN9K3j8t_Vo3I</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1385,17 +1420,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Senior .Net Developer8 - 15 yrsPune443+ ReviewsC#.Net.Net CoreEntity FrameworkPosted 1 week agoPosted 1 week ago</t>
+          <t>1691 Dotnet Job Vacancies In Pune</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1408,17 +1443,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/senior-net-developer-1678746?ref=sp&amp;jobPos=2</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZQHrOzAVq9r61qHO2mNgMGOP13tH3XS2xn-5xbwFqi0L_L86uBDHgl00dTuRMP7xAjDIrsGIqOBOa-83FpIsmU_b3bWrxvlM9k9nupMs8ImaWcfosbvQ0l2DNYMtVQH54xjrtdCr</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1427,17 +1463,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>.Net Developer5 - 8 yrsGurgaon/Gurugram.NetC#.Net CoreOOPSEntity FrameworkPosted 1 month agoPosted 1 month ago</t>
+          <t>Freshers Net Developer jobs in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1450,17 +1486,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-1673958?ref=sp&amp;jobPos=3</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEShwEB6zswFUY0xIJQjv-LeZTzzupzc_m9yFpXT51QoE_TL4OQEc7HD5J1lxEiXlR4DgD0cXjXqt310NyCUkawndX6p7HXFYZtzyQd5YXVQR9YQxYarbPwfWJ4R9mkYNrDg4iXUl7eLKcZzLepedqFAFuNO1oodL71Z9TXk9z351SAw--vhrRA0sQ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1469,17 +1506,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>.Net Developer - C#/ASP5 - 9 yrsHyderabad3.991+ Reviews.NetASPMultithreadingC#Posted 1 month agoPosted 1 month ago</t>
+          <t>Dot Net Developer Jobs In Pune</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1492,17 +1529,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-c-asp-1674099?ref=sp&amp;jobPos=5</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScAHrOzAVT8t0c2IVHC7G_EGpbcxnnJPye-xNyUsAPZluG7SOP1aQXOyId6hL8Wc-ebwgs5pewBpBHJkgIuF5vDN7AuU3EPbyy8UjJafgj8DGoff_MtfQPp2HTggvlC1BRjfsEj8QSUvJevvWX8_ZELk</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1511,17 +1549,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>.Net Developer4 - 6 yrs10-15 LPAGurgaon/Gurugram.NetC#.Net CoreSQL ServerASPPosted 1 month agoPosted 1 month ago</t>
+          <t>Dotnet Developer Jobs in Pune (1000+ Open Roles)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1534,17 +1572,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-1671544?ref=sp&amp;jobPos=6</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScgHrOzAV8zTS2vX4E4AqLpTMPZS6rsDoE8qZRoPOGSgV_0-0-SS74g3MUDT3VTqKxaAc1tvxCMKx7aO_3uQwwmwHTWXZqghA3cdZ1hDyTDl_RREBuebuBTs5wYwasbwYupcmuWCx_zJilPLj6kQEsPhN9g</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1553,17 +1592,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>.Net Developer - Distributed Backend4 - 6 yrsBangalore.NetC#ASPPosted 1 month agoPosted 1 month ago</t>
+          <t>400 Net Developer Job Vacancies in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1576,17 +1615,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-distributed-backend-1672423?ref=sp&amp;jobPos=7</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESfgHrOzAVHxk7pLd65-RI1Frhq0dQWMdaRUXshJ5cOIhA55C7oWC0P8aFoYbhofjhiWGjlND3OPQgMcVvm-paQHUvAPSzdVqa_l54Ha-y6cvj0VsoBD0yuQEwvB_EZa25uJO4okkbejs7KlmIwYbPoij0x-IwWmV2ZPSv7UT0tw</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1595,17 +1635,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Senior .Net Developer - Banking/Insurance Domain5 - 10 yrsMultiple Locations.NetC#Data StructureAlgorithmPosted 2 weeks agoPosted 2 weeks ago</t>
+          <t>Best NET Developer Jobs in Pune 2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1618,17 +1658,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/senior-net-developer-banking-insurance-domain-1677649?ref=sp&amp;jobPos=9</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESewHrOzAV4o8GwQAfkV7Wx2dSdT4A-khhbgqr1vl-XBth52G1VSh6BUgN7MTwYHZZFvlh8HGXwNIFemZq9RccTEmBHxXq9WEwGTQDXoESiklpYY3DPrYbOYI8JVlvyh4QEFJwULpRy3syDbvtJpcCCLlFN6Kwfe5Bc4F4Kw</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1637,17 +1678,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>.Net Developer - ASP/C#4 - 6 yrsGurgaon/Gurugram.Net.Net CoreC#SQL ServerPosted 1 month agoPosted 1 month ago</t>
+          <t>DOT NET Developer Jobs in Pune</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1660,17 +1701,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-asp-c-1671638?ref=sp&amp;jobPos=11</t>
-        </is>
-      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESgQEB6zswFYfpN4QsMFXhlHAvUe-x8cOoohXrTFhmO7B87MF6Bo3HR5jl3BUB5qGZp9Agf3XjzDhXVnihqVsend6JnGFomvqbQ1215-p1_Nv4EAszsdzKqIg8ll_fb2mNpk8U-UGb0BwLzU-5lPkgnKHXv8NHLohhid3hHgp0byanIhI</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1679,17 +1721,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>.Net Developer - C# Programming8 - 20 yrs20-25 LPAMultiple LocationsMay work from homeC#.NetSDLCSystem DesignPosted 1 month agoPosted 1 month ago</t>
+          <t>152+ .Net Jobs in Pune | .Net Job openings in Pune</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1702,17 +1744,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-c-programming-1671136?ref=sp&amp;jobPos=12</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZwHrOzAVfMGpfuI9EJ7QlubT2utDtOk80ImM6BlfiPtuOY5bCUy11eEf0juoGZb30PBzled4RgDQLafxzQ5jyTVmykco96g8aV_1NBhlZeX8vzfpRecFqQupWjiZfv3weLx64taHbmE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1721,17 +1764,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>.Net Developer - C#/AngularJS5 - 8 yrsBangalore.Net.Net CoreAngularJSSQL ServerC#ASPTypeScriptFull Stack+3Posted 1 month agoPosted 1 month ago</t>
+          <t>1691 Dotnet Job Vacancies In Pune</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1744,17 +1787,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-c-angularjs-1670525?ref=sp&amp;jobPos=15</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZQHrOzAVifbfAHUTNd18716eu3lmXSOa5wgYmJVMNbOHWsKIuWKEVzQyi6t0h0wVsEGEI7CV8nNm_-6z0ULjrZkWQaiGqBZYdz-4xif4C3p4fkG4lIA2blT5sRHELRa6AKCyOpHU</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1763,17 +1807,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>.Net Developer - C#/WPF5 - 8 yrsBangalore.Net.Net CoreC#WPFMultithreadingC+++1Posted 1 month agoPosted 1 month ago</t>
+          <t>Freshers Net Developer jobs in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1786,17 +1830,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-c-wpf-1670227?ref=sp&amp;jobPos=16</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEShwEB6zswFQ-pwiWo2DjkDoF4r4tOP14tD1K9UhqSoLZNIZ0B-98O12J1lTIxbLwh7pOD-_Eah1u086s5P3_hWb8bPjN0CTq42VevG2oVqR5CI6NidwxTsX6YKm-dSWcoEWdOSer8jxiGOJ3eN2vpvUsuU-nE2uhoxKcDk555R7xBz2lQb03zA5c</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1805,17 +1850,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>.Net Developer5 - 7 yrsMumbai.Net.Net CoreC#ASPPosted 1 month agoPosted 1 month ago</t>
+          <t>Dot Net Developer Jobs In Pune</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1828,17 +1873,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-1667585?ref=sp&amp;jobPos=17</t>
-        </is>
-      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScAHrOzAVJ7B3Ecp0nhil0eQCJnDTO2CcDLtWKTLXZ5KVsl0TWsf_XRKXL3sTCBivIATIG0SFsHL71BgmUfE6T6JsIELpd2o71lmB3xdmpIsouXUHjwHgDOrR87uSWnBxyvjYm9qkPcHycKh87GsWXvw</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1847,17 +1893,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>.Net Developer - ASP/MVC5 - 10 yrsBangalore4.324+ Reviews.NetBackend ArchitectureASPMVC.Net CoreC#+1Posted 1 month agoPosted 1 month ago</t>
+          <t>Dotnet Developer Jobs in Pune (1000+ Open Roles)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1870,17 +1916,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/net-developer-asp-mvc-1669727?ref=sp&amp;jobPos=18</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEScgHrOzAVSkGEzsMtp8TXZbZAb_qL5atmzw2pWslCrFriWozaSyuz8CwDyqMqujfm5tuqZuXKC-chYGdtbKQ8AY-jhPXlV2dwLcy95TT4bwnmm_fHeW9FladdLQZ2H2GURbZKWEprcpguFvwxEqMy3L4jBA</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1889,17 +1936,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Senior .Net Developer - C#/React.js8 - 12 yrsBangaloreC#.NetOpenAI.Net CoreReact.jsAngularJSFull Stack+2Posted 1 month agoPosted 1 month ago</t>
+          <t>400 Net Developer Job Vacancies in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>www.hirist.tech</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1912,17 +1959,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>https://www.hirist.tech/j/senior-net-developer-c-reactjs-1673568?ref=sp&amp;jobPos=20</t>
-        </is>
-      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESfgHrOzAVP9F5SWMN9UzFtAbVI3cPCBBaEfxN6_STK0eCyhYGHCvUFUGktoYLYy5l-nTUd8J2YXpMWHjgowhTAU_N-k_LgOoigEGARg2grD6MeD5NFxYz6wXm_HaOdFUzYPMA5wrWXjchBmHjY8JN0Ngdl8yyhrZdpecRDtFolw</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1931,17 +1979,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>.Net developer jobs pune indiawork from home</t>
+          <t>Best NET Developer Jobs in Pune 2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1954,17 +2002,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntr3hdahkGMqLucgtY6Jy5syj3Vfw:1792763564023&amp;q=.Net+developer+jobs+pune+india+work+from+home&amp;sa=X&amp;ved=2ahUKEwjPg5nbpNCXAxWrPDQIHeCdOQoQ1QJ6BAhQEAE</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESewHrOzAVrxDhXN6maso92KWpL_ET3mh9ifwM8yUqfvjbjoy6MOpiAqTs782bA0QPuAruAFPK4Y-iXdKb6UvbtzL9-vYecqJ19QEEX-5Cyuv8kUu91E3J4USgdVTkNl3MgRGGi_jFmdVf8zIAWhe9tv6cI8jyod_npVVHMA</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -1973,17 +2022,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>.Net developer jobs pune indiasalary</t>
+          <t>DOT NET Developer Jobs in Pune</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1996,17 +2045,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntr3hdahkGMqLucgtY6Jy5syj3Vfw:1792763564023&amp;q=.Net+developer+jobs+pune+india+salary&amp;sa=X&amp;ved=2ahUKEwjPg5nbpNCXAxWrPDQIHeCdOQoQ1QJ6BAhFEAE</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESgQEB6zswFdudhOo5cnweZ06orX6XP4ryDAbF2IsdF3oOjLnnIXNpes69mhf5kRvB6D9_ObDtvS8QYV4hzz1lvNTQjhV1pcZkMJlBklG7FiYCsMe2uvdXU-Rbl_DKaotD7ysVAzdQYkuIB4OQNoypWxHxPH-VNHTcowdac9vE5JP_LHU</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2015,17 +2065,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.Net developer jobs pune indiafor freshers</t>
+          <t>152+ .Net Jobs in Pune | .Net Job openings in Pune</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2038,17 +2088,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntr3hdahkGMqLucgtY6Jy5syj3Vfw:1792763564023&amp;q=.Net+developer+jobs+pune+india+for+freshers&amp;sa=X&amp;ved=2ahUKEwjPg5nbpNCXAxWrPDQIHeCdOQoQ1QJ6BAhBEAE</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZwHrOzAV7d8LdqT4-tfcvnAErCi_jnUCpdbHiR65V8GpFQXpneR60HjPDUyWLxAvsYI4XWsznQryRWaSwDeoJ5EdY6Yrzpc7ML5KsXeldCK1Unng9ouc-WTCFDYWF9i48IViWpYRT7M</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2057,22 +2108,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Remote .NET developer Jobs (October 2026) - Arcarc.devhttps://arc.dev› Remote Jobs</t>
+          <t>1691 Dotnet Job Vacancies In Pune</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2080,17 +2131,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>https://www.google.com/goto?url=CAESXgHrOzAVCbvde7V6bcZamEnbtfGUTuWAq99dQ_R8mdXC928nv6yN-wrMH1bu01miGwU4GmiNJwl2z80pIeFtolO2raDITZO6uqe2EauJ6ceDs7B9PZEssNlVK1GC06k</t>
-        </is>
-      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZQHrOzAVwWo7E3dLcsZ1CfJcNMUi2y5pz6Mkfec3P_Ey0FLDEyutdF5Q2SIvOgs7fYphSiN7Sb7gf5lzg4ANdMDWUvInaPuiaj3nkGo9t16ONzdbu2TTrhPLzC6zh9loDesg_wj6</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2099,22 +2151,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Remote .NET Developer Jobs in 2027Wellfoundhttps://wellfound.com› role › .net-developer</t>
+          <t>Freshers Net Developer jobs in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2122,17 +2174,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>https://www.google.com/goto?url=CAESZgHrOzAVyc8HMJN3MWSlKIZslHsGeBbspMXA79hCfo3IdIorL9CaNt-i5R-8yJbiTzDzvQoNHhH3PLxTH7f_WVTNsEwgVRaShST2mnulfJiqc8I-oyLDJzXgUFQTPKXA1O6_0G-SCA</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEShwEB6zswFSC9FAkyiGZePcFCCtcdtekMG52E1mmigjlYUc9sZqh4Yu_bR7b3hjMy-h11YlCsrveQUvQGeIqiRCEaQN62tF763QGCvb7nJkTpCECxev6QsgmzDqq8goF1nLbFhLrUqc2X8z2H1RYHg6TJXJ6ZpJmqA7RvXqvh206vi8SKncgvh2o</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2141,22 +2194,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>.Net developer jobs remoteindia</t>
+          <t>.NET Developer</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>TradeLab</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2164,17 +2217,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+india&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhLEAE</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-tradelab-JV_IC2940587_KO0,13_KE14,22.htm?jl=1010255443346</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2183,22 +2237,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>.Net developer jobs remoteworldwide</t>
+          <t>.net developer</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2206,17 +2260,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+worldwide&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhiEAE</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-infosys-JV_IC2940587_KO0,13_KE14,21.htm?jl=1010288783634</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2225,22 +2280,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>.Net developer jobs remotesalary</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Isar Systems</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2248,17 +2303,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+salary&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhlEAE</t>
-        </is>
-      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-isar-systems-JV_KO0,13_KE14,26.htm?jl=1009834125478</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2267,22 +2323,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>.Net developer jobs remotepart time</t>
+          <t>ASP.NET Developer</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>www.google.com</t>
+          <t>Bizupon</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Noida</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2290,17 +2346,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>https://www.google.com/search?sca_esv=0f046cdf8b4ca31a&amp;sxsrf=APpeQntjT_xCuIFaQ6JavNbiqzkgWfjULg:1792763563130&amp;q=.Net+developer+jobs+remote+part+time&amp;sa=X&amp;ved=2ahUKEwiJuuLapNCXAxW0EUQIHXrZBa0Q1QJ6BAhmEAE</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/asp-net-developer-bizupon-JV_IC4477468_KO0,17_KE18,25.htm?jl=1010296501663</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2309,22 +2366,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.Net Developer</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Digitup</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Gurgaon</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2332,17 +2389,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=8da132067a94c560&amp;bb=Hcx10gWOKryWGOh2y_7EE5QpFoqHsQNuAuapk5HKINXEnKcTUmVFaXzvbQvxrEBRoVYmPzjYtQu4LQfDtMK-RX-wd96d1rg33Twkql-aMnhs3Rp-VB7jBsEL9jBg_dlZ&amp;xkcb=SoCa67M2d0pPouz4BJ0LbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-digitup-JV_IC2921225_KO0,13_KE14,21.htm?jl=1010012158900</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2351,22 +2409,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>.net Developer- Windows Application Only (3-6 Yrs)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>TechnologiesIndia.com</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2374,17 +2432,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=006a32d5fe51635c&amp;bb=Hcx10gWOKryWGOh2y_7EE-Q8MMWd47rzMJebH_pyGCgl25D2AG3yEYhtEzy_fKCuMJ-uT7MdXCghLWgIh4bQ2r8BN9gy7egXBE5NRJeq5AbiYUysj7Ims9AcEdG81-48&amp;xkcb=SoAu67M2d0pPouz4BJ0KbzkdCdPP&amp;fccid=3d3123a1ac04ce14&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-windows-application-only-36-yrs-technologiesindia-com-JV_KO0,45_KE46,67.htm?jl=1008354378963</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2393,22 +2452,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Glassdoor</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Senior .Net Developer</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Luxoft</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2416,17 +2475,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=766ea748f5354651&amp;bb=Hcx10gWOKryWGOh2y_7EE33U3WPWSpyth_0atSPz4CoA6hKMgDIJ4uQuzvJRiXRX9YwQsz3x6b6r8fwHZ3FhY0y1-Hg2OFjIn30MG-IeFNOdCzBrVuGBaFayv9Cxh1d3&amp;xkcb=SoCz67M2d0pPouz4BJ0JbzkdCdPP&amp;fccid=99b9b1212188b67d&amp;cmp=Rosemallow-technologies&amp;ti=.NET+Developer&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.glassdoor.co.in/job-listing/senior-net-developer-luxoft-JV_KO0,20_KE21,27.htm?jl=1010287249096</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2435,22 +2495,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Work From Home Net Developer jobs in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2458,17 +2518,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=f04131cb17a8aa32&amp;bb=Hcx10gWOKryWGOh2y_7EE5vvfVvz3QB7f1yBYqIiMzHnyMGgVbdj8OVT84YYsdrmYutgCYqSGsPBmhfbl5BEFRuTZYgRwwd8kQTeFh2Sv5qZqDagoiij9rSgFGazPMKe&amp;xkcb=SoAH67M2d0pPouz4BJ0IbzkdCdPP&amp;fccid=7a162ca462563282&amp;cmp=Senwell-Solutions&amp;ti=.NET+Developer&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESjQEB6zswFWNewlIpG1flTMTMmShykZZJKosQiLGxlqGjgQ5GoXtBqZVUBJ6Kn9jLdPjvVJBa7_VAxaJzqXVHHPTBeyn4lM0JmMEm69t91yLEcNOqvxFtciC7TRyfBWUCaxub7RIiDTE6ogIudN7AZJCkP-QipqDrHedmNJZFutyE9Sl-YEHw5IPV2dkrgFA</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2477,22 +2538,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>32837 Dot Net Developer Job Vacancies In India Remote</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2500,17 +2561,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=d9afc88f5c049c6d&amp;bb=Hcx10gWOKryWGOh2y_7EE-rPlnHqhTOkkEH3_Mt9T34F3rY0AcavGqyGocIVQlisQGdJTy3IIUxYGOR5yFYj6DCeFktPR8tgnpB_Q0ArATrQV909VPuf_8JEHIv9cQeA&amp;xkcb=SoCJ67M2d0pPouz4BJ0PbzkdCdPP&amp;fccid=1f5c7702a1640572&amp;cmp=Steerlean-Consultancy-Services-Pvt.-Ltd.&amp;ti=.NET+Developer&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESeAHrOzAVy8cD8DWHme0Z8qLiKoHTOphhwGwaCSk-_1toKUHsBrGFby0hO26_XHuAvyMUcxwPQwWVl45bKbnlkM87scKGy8ci84wjy2jWST9jPVIz64kmHDMFrdKK20FV-tfZ6IzqUlPQxL8a3SAJ66nfBkCTxpC_xw</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2519,22 +2581,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>86 Work From Home Net Developer jobs in India</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2542,17 +2604,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=218f0f4a6447640b&amp;bb=Hcx10gWOKryWGOh2y_7EE3ChwAOoQd1Apv_Tssmn-8clmxgZXb-nw5fye9jpEhNm5gj1GVEA3H4iev9qBb6dye9a_SAgGyBBGYZO_BCLf7j39T8xV_DBHv4iFBBdT-Ui&amp;xkcb=SoA967M2d0pPouz4BJ0ObzkdCdPP&amp;fccid=15f3dea53ebe3c30&amp;cmp=Countless-services-private-limited&amp;ti=.NET+Developer&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESeQHrOzAVlcC_WwQ-XunpDV5Se1s2pD8iQDcuCdDcnrhlFmYY7OgXzNXV8K07gBUN59MGJXPfOSiHsCqxMTlQqnta7yq4ryRf6BQNYsnmzJXZQKNBfYC1pZ6PB0aLy9xpB4Lhvlj6HIHO3ovQtFn9C2gnPxQ0sffSX7U</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2561,22 +2624,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote .NET developer Jobs (October 2026) - Arc</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2584,17 +2647,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=566bdc09a50bcd32&amp;bb=Hcx10gWOKryWGOh2y_7EE7lXIprlQrgW94vy17jdL0rjrqS0gyZhQUksZnmPUMq3neQBzllr0C08pm1A2lvu-6Y4r72YXhbC3l538Z7To6RyNn0g0SlZ3pxmysVNxBVO&amp;xkcb=SoCg67M2d0pPouz4BJ0NbzkdCdPP&amp;fccid=c3d73a6fd53e8543&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESXgHrOzAVnl5Re3SS1PXeMxyTAdxp0ujH540PQCVO_fniJBu3k2jm4tQVcmw2zlWmsQWYwa5WIPnRaARWzGYPaEepJL5QBm7xx3SetwVUA76DHPl2Ys0gWUmndp_9GmQ</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2603,22 +2667,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Work from Home Dot NET Jobs in Pune</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2626,17 +2690,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=1782c21af7e0df75&amp;bb=Hcx10gWOKryWGOh2y_7EE6FqiodHdkZehui-OyBUzcr4L82Th7_uuIMDXloyiJNtCEvO7i8n_l6FsU2OFASDGY_5hUEmCoGhYKCctLi0Ng-qYnl7JQ9Fs9drFO4Siity&amp;xkcb=SoAU67M2d0pPouz4BJ0MbzkdCdPP&amp;fccid=74e36d81c894b4b7&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESawHrOzAVNA52BSlraXrbQURSsUT259ICR5DWAAHnHYYizkKg9NZrxQTy2MFtHEUfaRdj9Vifi12M-cSl7_x26mpJJYuYAJbRGA2xADIneDAZnqaryLm2efEIBy97KE1j4T22kwVV_I3oBthk</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2645,22 +2710,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>28 Net developer remote work jobs in Pune - Glassdoor</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2668,17 +2733,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=f6f2cf53a58a0fad&amp;bb=Hcx10gWOKryWGOh2y_7EE8eB_y_GBR24v-O0QJ7AlMWIK_vn1XgBk5LzOcgPLpSVzhst_I6baR4GW0jme5dEiKtiyZU32Z-pPRLGbhUKmE0W6qOxNUsGBmaRoMQ7Jo0p&amp;xkcb=SoD967M2d0pPouz4BJ0DbzkdCdPP&amp;fccid=464e2ee7fbea2edc&amp;cmp=SphereGen-Technologies&amp;ti=Senior+Developer&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESnwEB6zswFaS8YZgKKsyB2pAcbfkXYP0u3nvTheWGBnHn-jVRjlAwgYZk72dpLJlSS8Q-roOokMqubn9jrNGIPDGiZBa5UNHFv-id1VfmKAzxxBdKAmK9e41gbGYH9yDQo6nFX5kn5sT0VR8j-pFpQXY3uaXKV6hdYgDH-VPl-Am5Nhy_cwomsBTdPZDqZvaHzUdRJg2yLq_QoK3s2vL5J3I</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2687,22 +2753,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote net developer jobs in Pune, Maharashtra</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2710,17 +2776,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=79e3a0117be104c0&amp;bb=Hcx10gWOKryWGOh2y_7EE5qFmL_xhzR1S3W6gmsAapVCd0gLlN8gIewNczww7wyqtN2Rlv45PS4NSKOlb40aSXq5yr5zIyXZ7dAM_FrMZwBFGv0qTGXJDJwMtQY8hyPS&amp;xkcb=SoBJ67M2d0pPouz4BJ0CbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAEShQEB6zswFQxS-JhM6pmeyzMI_VIPLyLMe8oUAUXTH3bOGLvnILK8Yn42Cf3EM0wTIRXXnJzTlnPR8ES132waHEhwqhZfStx-ghED77bJK6j9Al-TaZ0d7UGVVO7AyovHuCrdqPfRFGvocQsrfHqlnDtqtZYxH_miq6zrOZQ_FzYiU5Gm2nmE</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2729,22 +2796,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote .NET Developer Jobs in 2027</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Google result</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2752,17 +2819,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=807e439b26cfd6ac&amp;bb=Hcx10gWOKryWGOh2y_7EE-uwu6I-hyrCsvwTNvhgXkOyb7jbpJw_xiI3QKJvsC7n1Asc3GT7ijAuKUsO4RchwkkKxNPYbV8B-3KdY99neorIfc-7OFj3k7I7tyM6RFE2&amp;xkcb=SoDU67M2d0pPouz4BJ0BbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://www.google.com/goto?url=CAESZgHrOzAVs-fmjTzUsmZ8jXHyLYo04GUzShCuB1ubHsJ5iFf29kQRyhsGdysPZeHMSnBPgK-E2MgQZgWv3yFfcmOdu5wh14-7Vw97O1ltL3Zm23fGuudqPa1lqYuqf8r8k0PTLjgMCQ</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2794,17 +2862,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=e87d802dead8432d&amp;bb=Hcx10gWOKryWGOh2y_7EE4rbgza9sJw-7z94nnZKfNakGTsb-0TYL_edkDm2AXIfDKHh4vnMqk_hL41NNnefjbU3AsYK_Y7-dKDYRVx45yJxvlSnbTEs92X9OvzMFp1o&amp;xkcb=SoBg67M2d0pPouz4BJ0AbzkdCdPP&amp;fccid=2fad1b49105da4f2&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.indeed.com/rc/clk?jk=8da132067a94c560&amp;bb=_ewUAmqf8cGRwxOLZ_naAA4811Sokwi6HrB_-bOeskoSFIc7f0h0ToDnICJL8dk4S5TKZdhDVjgZMvzjcigvfli5CEUfrRjsb9hfRsk129DOkkZmRPHb8eq0Cz8G7QOE&amp;xkcb=SoBo67M2d0ipvBT4BJ0LbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2836,17 +2905,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=df1aa1127172a51f&amp;bb=Hcx10gWOKryWGOh2y_7EE-uwu6I-hyrCTFaHZ3myIXZTIrLK3VrlVPqPmqFF628DY7z4p9mwpRRXwTRmAOVx8Kd5tAzKbORRIPCLgGjvjakyaYPYIZpf_bhUpUU9G0eJ&amp;xkcb=SoDu67M2d0pPouz4BJ0HbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.indeed.com/rc/clk?jk=006a32d5fe51635c&amp;bb=_ewUAmqf8cGRwxOLZ_naAMzNhwOKtC7NghO9hT7TJEToXowwnOJmoWwMHTbd7jmGFbgsnJLEnQXm7MIZrIb1_7aVUL_W5Qd196vBR1G7FsfKsMaWQNM_7jIMzYljNG-E&amp;xkcb=SoDc67M2d0ipvBT4BJ0KbzkdCdPP&amp;fccid=3d3123a1ac04ce14&amp;vjs=3</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2878,17 +2948,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=2aa74008fc68d77c&amp;bb=Hcx10gWOKryWGOh2y_7EE1W7ljh1w4ER_EHxQg9LUDnU39S6q_zDyFM9qkEuVWBJH__NCdnBj_n0q5Ow1HrS493eYeqmeN7CQETpmOisW7fEkW55Eb60mbWQSPgmLLlh&amp;xkcb=SoBa67M2d0pPouz4BJ0GbzkdCdPP&amp;fccid=b90433ed96d63887&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.indeed.com/rc/clk?jk=766ea748f5354651&amp;bb=_ewUAmqf8cGRwxOLZ_naAFqWGP4BbjRqZYFk5L5tGyTF9Nj2tFVGTZHao9GCl9CscWsALEqAOKRAfAHEk9RpkZJsACEZgBX9jz4dm3XFKYin75H259VtzASE53jXjrhU&amp;xkcb=SoBB67M2d0ipvBT4BJ0JbzkdCdPP&amp;fccid=99b9b1212188b67d&amp;cmp=Rosemallow-technologies&amp;ti=.NET+Developer&amp;vjs=3</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2920,17 +2991,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/viewjob?jk=cdef0123456789ab</t>
-        </is>
-      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.indeed.com/rc/clk?jk=f04131cb17a8aa32&amp;bb=_ewUAmqf8cGRwxOLZ_naAA7ICOt7cDm_sssqxfWS-1kyqONJyo0TA8JxK1hyh_lC640BQ6q9Bx0Q-oBuEHn4KV8z0BncTpB1PyW2p-nDVaKtK_soVY3BSuKV2eeSXgP6&amp;xkcb=SoD167M2d0ipvBT4BJ0IbzkdCdPP&amp;fccid=7a162ca462563282&amp;cmp=Senwell-Solutions&amp;ti=.NET+Developer&amp;vjs=3</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2962,17 +3034,18 @@
           <t>5-8 years</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>https://in.indeed.com/rc/clk?jk=b212ad1b8a056e3a&amp;bb=Hcx10gWOKryWGOh2y_7EEwK02jMB57x59l-xgPHPMV2drIXGa2bp3gJ5CJHFYHsOPr41bBcMHd0QQubsVlb5zoeMefIduFhDtS8X9yQzo6EDlXyXV8pVvBv-zfZYwrTI&amp;xkcb=SoDH67M2d0pPouz4BJ0FbzkdCdPP&amp;fccid=105ecfd0283f415f&amp;vjs=3</t>
-        </is>
-      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Refer to Apply Link</t>
+          <t>https://in.indeed.com/rc/clk?jk=d9afc88f5c049c6d&amp;bb=_ewUAmqf8cGRwxOLZ_naAMTveVICCDy0UvlKPZifSx67JsaFotMlla43gZNsQUbFYt-4J1difXgoGG8YaiTbNb4Kulyu4baZ_CXKOLnDEwe3aTPFt37dzbBdSeKQQk3N&amp;xkcb=SoB767M2d0ipvBT4BJ0PbzkdCdPP&amp;fccid=1f5c7702a1640572&amp;cmp=Steerlean-Consultancy-Services-Pvt.-Ltd.&amp;ti=.NET+Developer&amp;vjs=3</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>
@@ -2981,40 +3054,901 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=566bdc09a50bcd32&amp;bb=_ewUAmqf8cGRwxOLZ_naABI8rBcndX_aNoS9330G0W_z7nmHS_166bJEGy7s-uCDelMai6PYOJYbnvLgY8PMGWMT-hV1dH-3xlyLNezKUlRu9nFLh7CiCIVonmjFfw9s&amp;xkcb=SoDP67M2d0ipvBT4BJ0ObzkdCdPP&amp;fccid=c3d73a6fd53e8543&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=f6f2cf53a58a0fad&amp;bb=_ewUAmqf8cGRwxOLZ_naAAoJLBauahaS3Etimp7nd0z0Ebg-t6Pe7ofcMReoup_Tqq3lEv37HK2yhPxtJQoXrQJ9B_ojB6O1N1n6rTHmJbL_dCmmQMf_H0sew922AVy9&amp;xkcb=SoBS67M2d0ipvBT4BJ0NbzkdCdPP&amp;fccid=464e2ee7fbea2edc&amp;cmp=SphereGen-Technologies&amp;ti=Senior+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=58893641e84162d6&amp;bb=_ewUAmqf8cGRwxOLZ_naABxTa0kAvggdVzgEaDQnxS0YRF1ep5lVIxf7vLXXAiIs-XRHo7darbTtDmIbp8ZAC_XSBXGrNje8tGgQ0zF0RcH_XhCRlMv_OGlc66qjmJ83&amp;xkcb=SoDm67M2d0ipvBT4BJ0MbzkdCdPP&amp;fccid=a0563012c42115b5&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=218f0f4a6447640b&amp;bb=_ewUAmqf8cGRwxOLZ_naAJM1dnnkSoAnWlml9NUQyxDDW6YnV7l5JqyxIbmCIFhNBR7OhRPozYWFp8f-4s9_T0Cx_r75FcAbR4bn0zF4tYnBQ3X01wQY_FQufm6kUpZ3&amp;xkcb=SoAP67M2d0ipvBT4BJ0DbzkdCdPP&amp;fccid=15f3dea53ebe3c30&amp;cmp=Countless-services-private-limited&amp;ti=.NET+Developer&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=1782c21af7e0df75&amp;bb=_ewUAmqf8cGRwxOLZ_naAB-MQFAaHi9iSvZDZlR72sePPg-eKDBzCUXKALRCJ61KtHNzclo7bCzkPz-TSJOHuA_a7rLlSoiVtlKTdqwyd8s1w9eoJGkLQsmblc4EwbOd&amp;xkcb=SoC767M2d0ipvBT4BJ0CbzkdCdPP&amp;fccid=74e36d81c894b4b7&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=123456789abcdef0</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=807e439b26cfd6ac&amp;bb=_ewUAmqf8cGRwxOLZ_naANfHduWWn-o9t6KHmeo-nJ_a9GDm7NIvE2RlImjMRm3YxjRPLD6rWc7l4Um5X2LOo85jEPq4dUHfgMBFl1YXgbxJ9y6dL8ZlMm6r8KBsJ0Hw&amp;xkcb=SoAm67M2d0ipvBT4BJ0BbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=79e3a0117be104c0&amp;bb=_ewUAmqf8cGRwxOLZ_naAHweyzzcJ7S-SQiHZqg24RCZ9h-mnedyUWQ_YZn7IOEIixPsSdMZfK--c-xIwvxwfddA2E3scmgPLKkZp1sPvfYx1NH-RlcmQCq4ujerNQXd&amp;xkcb=SoCS67M2d0ipvBT4BJ0AbzkdCdPP&amp;fccid=8d25321c1defe73f&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=e87d802dead8432d&amp;bb=_ewUAmqf8cGRwxOLZ_naADwTfNwoY6QoNGsSA3LmsE1bMJbsxUg9guuRgKDIcyYOCOapKP223nO1rqL5ZQFIaKqvkvATh0EOLdOoTt_xba6GtDIF-SUC7KnBTveE0Hbc&amp;xkcb=SoAc67M2d0ipvBT4BJ0HbzkdCdPP&amp;fccid=2fad1b49105da4f2&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=cecf6a9987df2156&amp;bb=_ewUAmqf8cGRwxOLZ_naAB-MQFAaHi9i_kgjlOfyqgsjVl2DvHcC_U8TQbwHW-G7Y-01UgSCxHrl1cOyHuQRBDnam1XGgsZOqdi-ggaFiZ-fr6oYr1Ev512Jqg0KoTRp&amp;xkcb=SoCo67M2d0ipvBT4BJ0GbzkdCdPP&amp;fccid=afe30394bfba1470&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/rc/clk?jk=df1aa1127172a51f&amp;bb=_ewUAmqf8cGRwxOLZ_naANfHduWWn-o9urkCn_M1zUWwJqo8s7NdBaBA59sUUZ1ZMtbvwke3Fa31K2rVdTQ8pdB_FX3S1HcbfkkbO66lWuH04dDjZdZjOh6t4hZpkOsF&amp;xkcb=SoA167M2d0ipvBT4BJ0FbzkdCdPP&amp;fccid=03cacc905f5db444&amp;vjs=3</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>Glassdoor</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ASP.NET Developer</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Navare Solutions Pvt. Ltd</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Cochin</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/asp-net-developer-navare-solutions-pvt-ltd-JV_IC2887994_KO0,17_KE18,42.htm?jl=1010304480249</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Junior .Net Developer</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Aeon Software</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/junior-net-developer-aeon-software-JV_KO0,20_KE21,34.htm?jl=1010294023347</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>.NET Developer</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Propel Technology Group</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-propel-technology-group-JV_IC2833209_KO0,13_KE14,37.htm?jl=1010226779700</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>.NET Developer</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>India Insure</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Hyderābād</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-india-insure-JV_IC2865319_KO0,13_KE14,26.htm?jl=1009562194926</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Software Engineer (.Net Developer)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>McIver Software LLP</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Ahmedabad</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/software-engineer-net-developer-mciver-software-llp-JV_IC2935226_KO0,31_KE32,51.htm?jl=1010277252578</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Sr .Net Developer</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>GlobusSoft</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/sr-net-developer-globussoft-JV_KO0,16_KE17,27.htm?jl=1007982852083</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>.NET Developer</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Great Place IT Services</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Nāgpur</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-great-place-it-services-JV_IC2951950_KO0,13_KE14,37.htm?jl=1009037945795</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Senior .Net Developer</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Cognet Corp</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/senior-net-developer-cognet-corp-JV_IC2833209_KO0,20_KE21,32.htm?jl=1010297812803</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
         <is>
           <t>.Net Developer</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Realizer Technologies</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Kh Infinite Possibilities</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>5-8 years</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>https://www.glassdoor.co.in/job-listing/net-developer-realizer-technologies-JV_KO0,13_KE14,35.htm?jl=1007531044310</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Refer to Apply Link</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-kh-skill-academy-JV_KO0,13_KE14,30.htm?jl=1009347845690</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>.NET Developer</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Tech extensor</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>5-8 years</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/net-developer-tech-extensor-JV_KO0,13_KE14,27.htm?jl=1010047987391</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Refer to Apply Link</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
         <is>
           <t>permanent</t>
         </is>

</xml_diff>